<commit_message>
data: update prices 2026-09-20
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -517,6 +517,62 @@
       <c r="F3" t="inlineStr">
         <is>
           <t>2026-09-19T20:25:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>7669</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-09-20T17:09:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>459.6</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-09-20T17:09:27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: update prices 2026-09-21
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -573,6 +573,62 @@
       <c r="F5" t="inlineStr">
         <is>
           <t>2026-09-20T17:09:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>7709</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-09-21T20:27:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>459.5</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-09-21T20:27:41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: update prices 2026-09-23
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -632,6 +632,118 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>7752.33</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-09-22T20:37:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>460</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-09-22T20:37:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>7752.33</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-09-23T19:01:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>459</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-09-23T19:01:55</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-09-24
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -744,6 +744,62 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>7719</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-09-24T19:37:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>458</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-09-24T19:37:08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-09-25
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -800,6 +800,62 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>7719</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-09-27T23:12:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>457.25</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-09-27T23:12:10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-09-28
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -856,6 +856,62 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>7735.67</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-09-28T22:41:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>457</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-09-28T22:41:32</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-09-29
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -912,6 +912,62 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>7752.33</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-09-29T20:36:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>460</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-09-29T20:36:10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-09-30
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -968,6 +968,62 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>7685.67</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-09-30T20:04:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>456</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-09-30T20:04:57</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-01
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1024,6 +1024,62 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>7702.33</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-10-01T19:11:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>435</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2026-10-01T19:11:07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-02
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1080,6 +1080,62 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>7702.33</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-10-02T20:18:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>432.5</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-10-02T20:18:22</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-03
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1136,6 +1136,62 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>7702.33</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-10-03T20:12:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>446.5</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-10-03T20:12:35</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-04
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1192,6 +1192,62 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>7702.33</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-10-04T16:11:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>446.5</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-10-04T16:11:55</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-05
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1248,6 +1248,62 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>7702.33</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-10-05T19:40:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>446.5</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2026-10-05T19:40:27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-06
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1304,6 +1304,62 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>7702.33</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2026-10-06T18:23:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>440</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-10-06T18:23:16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-07
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1360,6 +1360,62 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>7702.33</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2026-10-08T22:48:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>435</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2026-10-08T22:48:14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-08
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1416,6 +1416,62 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>7402.33</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-10-08T22:49:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>435</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2026-10-08T22:49:37</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-09
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1472,6 +1472,62 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>7392.33</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2026-10-09T17:14:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>441</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2026-10-09T17:14:15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-12
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1528,6 +1528,62 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>7319</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2026-10-12T20:35:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>438.5</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2026-10-12T20:35:09</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-13
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1584,6 +1584,62 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>7190</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2026-10-14T17:14:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>450</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2026-10-14T17:14:41</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-14
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1640,6 +1640,62 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>7166.67</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>2026-10-14T17:15:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>450</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2026-10-14T17:15:19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-15
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1696,6 +1696,62 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>6669</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2026-10-16T21:08:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>461.5</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2026-10-16T21:08:46</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-16
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1752,6 +1752,62 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>6652.33</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2026-10-16T21:09:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>457.5</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2026-10-16T21:09:20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-19
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1808,6 +1808,62 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>6076.75</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>2026-10-19T19:18:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>455.5</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2026-10-19T19:18:11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-20
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1864,6 +1864,62 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>6076.8</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2026-10-29T21:27:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>444</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>2026-10-29T21:27:14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-21
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1920,6 +1920,62 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>5776.8</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>2026-10-29T21:28:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>444</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>2026-10-29T21:28:26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-22
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1976,6 +1976,62 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>5714.3</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>2026-10-29T21:29:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>442.5</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>2026-10-29T21:29:04</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-23
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2032,6 +2032,62 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>5714.3</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>2026-10-29T21:29:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>453</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>2026-10-29T21:29:50</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-26
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2088,6 +2088,62 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>5614.3</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>2026-10-29T21:30:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>447.5</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>2026-10-29T21:30:34</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-27
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2144,6 +2144,62 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>5564.3</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>2026-10-29T21:31:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>446.5</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>2026-10-29T21:31:10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-28
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2200,6 +2200,62 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>5551.8</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>2026-10-29T21:31:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>446.5</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>2026-10-29T21:31:48</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-29
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2256,6 +2256,62 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>5551.75</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>2026-10-29T21:32:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>446.5</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>2026-10-29T21:32:21</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update prices 2026-10-30
</commit_message>
<xml_diff>
--- a/data/commodity_prices.xlsx
+++ b/data/commodity_prices.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F67"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2312,6 +2312,62 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>5344.25</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>CNY/T</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>2026-10-30T22:34:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Urea</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>449.5</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>USD/T</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Manual entry</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>2026-10-30T22:34:07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>